<commit_message>
Updated cellvalues in Excel Sheet using python
</commit_message>
<xml_diff>
--- a/Marks.xlsx
+++ b/Marks.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Grades" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Grades'!$A$1:$E$9</definedName>
@@ -459,7 +459,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Arjun</t>
+          <t>Teja</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Priya</t>
+          <t>Srinu</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C6" t="n">
         <v>75</v>

</xml_diff>